<commit_message>
Équipement : « Armure » devient « Manteau » (anglais : Coat)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/lexique.xlsx
+++ b/i18n/lexique.xlsx
@@ -147,7 +147,7 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pièces d’équipement : noms génériques choisis pour le site (Casque, Montre, Armure, Pantalon, Bague, Bâton / Helmet, Watch, Armor, Pants, Ring, Staff), car le jeu donne un nom différent à chaque pièce selon son niveau. « Veste » et « Canne » deviendront « Armure » et « Bâton » au branchement.</t>
+          <t xml:space="preserve">   Pièces d’équipement : noms génériques choisis pour le site (Casque, Montre, Manteau, Pantalon, Bague, Bâton / Helmet, Watch, Coat, Pants, Ring, Staff), car le jeu donne un nom différent à chaque pièce selon son niveau. « Veste » et « Canne » sont devenus « Manteau » et « Bâton ».</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.armure</t>
+          <t xml:space="preserve">game.bague</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
@@ -5483,24 +5483,19 @@
           <t xml:space="preserve">Pièce d’équipement</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Armure</t>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bague</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armor</t>
+          <t xml:space="preserve">Ring</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nom générique choisi pour le site (les noms du jeu changent selon le niveau de la pièce)</t>
-        </is>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nouveau nom FR (aujourd’hui « Veste » sur le site, changera au branchement)</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
@@ -5517,7 +5512,7 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.bague</t>
+          <t xml:space="preserve">game.baton</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
@@ -5525,19 +5520,24 @@
           <t xml:space="preserve">Pièce d’équipement</t>
         </is>
       </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bague</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bâton</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ring</t>
+          <t xml:space="preserve">Staff</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nom générique choisi pour le site (les noms du jeu changent selon le niveau de la pièce)</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nouveau nom FR (aujourd’hui « Canne » sur le site, changera au branchement)</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -5554,7 +5554,7 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.baton</t>
+          <t xml:space="preserve">game.casque</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
@@ -5562,14 +5562,14 @@
           <t xml:space="preserve">Pièce d’équipement</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bâton</t>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casque</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff</t>
+          <t xml:space="preserve">Helmet</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -5577,14 +5577,9 @@
           <t xml:space="preserve">Nom générique choisi pour le site (les noms du jeu changent selon le niveau de la pièce)</t>
         </is>
       </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nouveau nom FR (aujourd’hui « Canne » sur le site, changera au branchement)</t>
-        </is>
-      </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Talismans</t>
+          <t xml:space="preserve">Talismans, Équipement</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -5596,7 +5591,7 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.casque</t>
+          <t xml:space="preserve">game.manteau</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
@@ -5604,14 +5599,14 @@
           <t xml:space="preserve">Pièce d’équipement</t>
         </is>
       </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Casque</t>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manteau</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Helmet</t>
+          <t xml:space="preserve">Coat</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -5619,9 +5614,14 @@
           <t xml:space="preserve">Nom générique choisi pour le site (les noms du jeu changent selon le niveau de la pièce)</t>
         </is>
       </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nouveau nom FR (aujourd’hui « Veste » sur le site, changera au branchement)</t>
+        </is>
+      </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Talismans, Équipement</t>
+          <t xml:space="preserve">Talismans</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Espagnol : 10 termes confirmés par captures (Calefactor, Muro Indomable, Enchapado / Escudos fundidos, unités T12…)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/lexique.xlsx
+++ b/i18n/lexique.xlsx
@@ -1366,7 +1366,7 @@
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configura el nivel actual de tu Horno y el que quieres alcanzar.</t>
+          <t xml:space="preserve">Configura el nivel actual de tu Calefactor y el que quieres alcanzar.</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total edificios + Horno</t>
+          <t xml:space="preserve">Total edificios + Calefactor</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horno actual</t>
+          <t xml:space="preserve">Calefactor actual</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="H36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horno {id}</t>
+          <t xml:space="preserve">Calefactor {id}</t>
         </is>
       </c>
       <c r="I36" s="0" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="H98" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horno objetivo</t>
+          <t xml:space="preserve">Calefactor objetivo</t>
         </is>
       </c>
       <c r="J98" s="0" t="inlineStr">
@@ -6053,12 +6053,12 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horno</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Calefactor</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I4" s="0" t="inlineStr">
@@ -6793,12 +6793,12 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blindaje fundido</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Enchapado fundido</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I19" s="0" t="inlineStr">
@@ -7031,9 +7031,9 @@
           <t xml:space="preserve">Escudos fundidos</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
@@ -7404,12 +7404,12 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrenamiento de Infanterías Sublimes</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Entrenamiento de Infantería Sublime</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I32" s="0" t="inlineStr">
@@ -7454,9 +7454,9 @@
           <t xml:space="preserve">Entrenamiento de Lanceros Sublimes</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I33" s="0" t="inlineStr">
@@ -7746,9 +7746,9 @@
           <t xml:space="preserve">Flecha de Cristal</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I39" s="0" t="inlineStr">
@@ -8260,12 +8260,12 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muro indomable</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Muro Indomable</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I50" s="0" t="inlineStr">
@@ -8448,12 +8448,12 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Primeros Auxilios de Infanterías Sublimes</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Primeros Auxilios de Infantería Sublime</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I54" s="0" t="inlineStr">
@@ -8592,9 +8592,9 @@
           <t xml:space="preserve">Protección de Cristal</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I57" s="0" t="inlineStr">
@@ -8777,12 +8777,12 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Curación de Infanterías Sublimes</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Curación de Infantería Sublime</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Officiel — capture du jeu en espagnol (IMG_1340 à 1356)</t>
         </is>
       </c>
       <c r="I61" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Espagnol : pièces de déblocage T12 déduites des noms EN/FR, raretés validées
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/lexique.xlsx
+++ b/i18n/lexique.xlsx
@@ -140,7 +140,7 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ES : termes du jeu relevés sur tes captures en espagnol (IMG_1284 à 1339) ; ceux qui n’y figurent pas sont des propositions en jaune, à vérifier en jeu.</t>
+          <t xml:space="preserve">   ES : termes du jeu relevés sur tes captures en espagnol (IMG_1284 à 1356). Les 15 pièces de déblocage T12 (en jaune) sont déduites des noms officiels anglais et français, faute de source espagnole.</t>
         </is>
       </c>
     </row>
@@ -6395,9 +6395,9 @@
           <t xml:space="preserve">Legendario{x}</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -6447,9 +6447,9 @@
           <t xml:space="preserve">Mítico</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="I12" s="0" t="inlineStr">
@@ -6494,9 +6494,9 @@
           <t xml:space="preserve">Mítico{x}</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -6546,9 +6546,9 @@
           <t xml:space="preserve">Poco común{x}</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -6598,9 +6598,9 @@
           <t xml:space="preserve">Raro{x}</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -6650,9 +6650,9 @@
           <t xml:space="preserve">Épico</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="I16" s="0" t="inlineStr">
@@ -6697,9 +6697,9 @@
           <t xml:space="preserve">Épico{x}</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validé par toi</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I18" s="0" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I25" s="0" t="inlineStr">
@@ -7122,12 +7122,12 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yelmo sublime</t>
+          <t xml:space="preserve">Casco sublime</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I26" s="0" t="inlineStr">
@@ -7268,7 +7268,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
@@ -7696,12 +7696,12 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travesía sublime</t>
+          <t xml:space="preserve">Excursión sublime</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I38" s="0" t="inlineStr">
@@ -7931,12 +7931,12 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hombreras sublimes</t>
+          <t xml:space="preserve">Hombrera sublime</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I43" s="0" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I49" s="0" t="inlineStr">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I52" s="0" t="inlineStr">
@@ -8406,7 +8406,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I53" s="0" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I65" s="0" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I69" s="0" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I71" s="0" t="inlineStr">
@@ -9502,7 +9502,7 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposition — à vérifier en jeu</t>
+          <t xml:space="preserve">Déduit des noms officiels EN et FR (aucune source espagnole publique), modèle du jeu « … sublime »</t>
         </is>
       </c>
       <c r="I76" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Accueil : phrase de bas d'écran réduite à « Outil communautaire non officiel » (4 langues)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/lexique.xlsx
+++ b/i18n/lexique.xlsx
@@ -1360,22 +1360,22 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outil communautaire non officiel · Les données V1 sont isolées et versionnées pour audit.</t>
+          <t xml:space="preserve">Outil communautaire non officiel</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unofficial community tool · V1 data is isolated and versioned for auditing.</t>
+          <t xml:space="preserve">Unofficial community tool</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herramienta comunitaria no oficial · Los datos V1 están aislados y versionados para auditoría.</t>
+          <t xml:space="preserve">Herramienta comunitaria no oficial</t>
         </is>
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strumento non ufficiale della community · I dati V1 sono isolati e versionati per la verifica.</t>
+          <t xml:space="preserve">Strumento non ufficiale della community</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">

</xml_diff>